<commit_message>
Fix: deferred CARE pension should not keep growing at 1.5% real
Between retirement age and NHS claim age, the member is deferred, not
active. NHS 2015 Scheme deferred CARE pensions revalue at CPI only, not
the active member's CPI+1.5%, and this model already strips CPI out
throughout -- so real growth during that gap should be 0%, not the
1.5% real rate that was being applied. Only affects scenarios with a
deferral gap (retirementAge < nhsClaimAge); immediate-claim scenarios
are unaffected since the compounding term was a no-op there anyway.

Regenerated the deferred-claim test fixture and ground truth from the
corresponding spreadsheet fix.
</commit_message>
<xml_diff>
--- a/test/scenario_deferred.xlsx
+++ b/test/scenario_deferred.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="398">
   <si>
     <t>NHS + Private Pension Retirement Modeller — Product Spec (v0.1)</t>
   </si>
@@ -619,9 +619,6 @@
     <t>NHS 2015 Scheme + AP, before early retirement reduction (at claim age)</t>
   </si>
   <si>
-    <t>CARE pot stops accruing new service at your retirement age, then simply revalues (no new accrual) until your claim age</t>
-  </si>
-  <si>
     <t xml:space="preserve">  — early retirement reduction (ERRBO offsets this)</t>
   </si>
   <si>
@@ -1217,6 +1214,15 @@
   </si>
   <si>
     <t>For GPs, legacy 1995/2008 pension benefits keep growing in real terms (CPI + 1.5%, with a 1.5% floor) right up until you claim them, as long as you don't have a 5+ year break in NHS pensionable service. Officers get a similar link, but to current pay scales instead.</t>
+  </si>
+  <si>
+    <t>TOTAL ANNUAL INCOME FROM STATE PENSION AGE ONWARDS</t>
+  </si>
+  <si>
+    <t>The claim-age total above is a steady-state figure that never includes the State Pension if you claim your NHS pension before your State Pension Age — it treats that gap the same way forever, even after you actually turn State Pension Age. This row adds the State Pension back in for scenarios that claim early, showing your true steady income from State Pension Age onwards. If you already claim at or after State Pension Age, this is identical to the row above (State Pension is already included there).</t>
+  </si>
+  <si>
+    <t>CARE pot stops accruing new service at your retirement age. If you defer claiming past that (retirement age before claim age), you become a DEFERRED member — NHS Pensions revalues deferred CARE at CPI only, not the active member's CPI+1.5%. Since this model works in real terms with CPI already stripped out, that means no further real growth during the gap: the pot is simply held flat (in today's money) from retirement age to claim age.</t>
   </si>
 </sst>
 </file>
@@ -1812,60 +1818,60 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="3" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="40" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B3" s="40"/>
       <c r="C3" s="40"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>266</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="C5" s="36" t="s">
         <v>267</v>
-      </c>
-      <c r="C5" s="36" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="B6" s="37" t="s">
         <v>269</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="C6" s="38" t="s">
         <v>270</v>
-      </c>
-      <c r="C6" s="38" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="B7" s="37" t="s">
         <v>272</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="C7" s="38" t="s">
         <v>273</v>
-      </c>
-      <c r="C7" s="38" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="B8" s="37" t="s">
         <v>275</v>
       </c>
-      <c r="B8" s="37" t="s">
+      <c r="C8" s="38" t="s">
         <v>276</v>
-      </c>
-      <c r="C8" s="38" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1873,54 +1879,54 @@
         <v>117</v>
       </c>
       <c r="B9" s="37" t="s">
+        <v>277</v>
+      </c>
+      <c r="C9" s="38" t="s">
         <v>278</v>
-      </c>
-      <c r="C9" s="38" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="B10" s="37" t="s">
         <v>280</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="C10" s="38" t="s">
         <v>281</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B11" s="37" t="s">
         <v>283</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="C11" s="38" t="s">
         <v>284</v>
-      </c>
-      <c r="C11" s="38" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
+        <v>285</v>
+      </c>
+      <c r="B12" s="37" t="s">
         <v>286</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="C12" s="38" t="s">
         <v>287</v>
-      </c>
-      <c r="C12" s="38" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="B13" s="37" t="s">
         <v>289</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="C13" s="38" t="s">
         <v>290</v>
-      </c>
-      <c r="C13" s="38" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1928,197 +1934,197 @@
         <v>74</v>
       </c>
       <c r="B14" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="C14" s="38" t="s">
         <v>292</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
+        <v>293</v>
+      </c>
+      <c r="B15" s="37" t="s">
         <v>294</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="C15" s="38" t="s">
         <v>295</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
+        <v>296</v>
+      </c>
+      <c r="B16" s="37" t="s">
         <v>297</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="C16" s="38" t="s">
         <v>298</v>
-      </c>
-      <c r="C16" s="38" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="B17" s="37" t="s">
         <v>300</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="C17" s="38" t="s">
         <v>301</v>
-      </c>
-      <c r="C17" s="38" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="21" t="s">
+        <v>302</v>
+      </c>
+      <c r="B18" s="37" t="s">
         <v>303</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="C18" s="38" t="s">
         <v>304</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="B19" s="37" t="s">
         <v>306</v>
       </c>
-      <c r="B19" s="37" t="s">
+      <c r="C19" s="38" t="s">
         <v>307</v>
-      </c>
-      <c r="C19" s="38" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="B20" s="37" t="s">
         <v>309</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="C20" s="38" t="s">
         <v>310</v>
-      </c>
-      <c r="C20" s="38" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
+        <v>311</v>
+      </c>
+      <c r="B21" s="37" t="s">
         <v>312</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="C21" s="38" t="s">
         <v>313</v>
-      </c>
-      <c r="C21" s="38" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
+        <v>314</v>
+      </c>
+      <c r="B22" s="37" t="s">
         <v>315</v>
       </c>
-      <c r="B22" s="37" t="s">
+      <c r="C22" s="38" t="s">
         <v>316</v>
-      </c>
-      <c r="C22" s="38" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
+        <v>317</v>
+      </c>
+      <c r="B23" s="37" t="s">
         <v>318</v>
       </c>
-      <c r="B23" s="37" t="s">
+      <c r="C23" s="38" t="s">
         <v>319</v>
-      </c>
-      <c r="C23" s="38" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="21" t="s">
+        <v>320</v>
+      </c>
+      <c r="B24" s="37" t="s">
         <v>321</v>
       </c>
-      <c r="B24" s="37" t="s">
+      <c r="C24" s="38" t="s">
         <v>322</v>
-      </c>
-      <c r="C24" s="38" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="B25" s="37" t="s">
         <v>324</v>
       </c>
-      <c r="B25" s="37" t="s">
+      <c r="C25" s="38" t="s">
         <v>325</v>
-      </c>
-      <c r="C25" s="38" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
+        <v>326</v>
+      </c>
+      <c r="B26" s="37" t="s">
         <v>327</v>
       </c>
-      <c r="B26" s="37" t="s">
+      <c r="C26" s="38" t="s">
         <v>328</v>
-      </c>
-      <c r="C26" s="38" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="B27" s="37" t="s">
         <v>330</v>
       </c>
-      <c r="B27" s="37" t="s">
+      <c r="C27" s="38" t="s">
         <v>331</v>
-      </c>
-      <c r="C27" s="38" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="B28" s="37" t="s">
         <v>333</v>
       </c>
-      <c r="B28" s="37" t="s">
+      <c r="C28" s="38" t="s">
         <v>334</v>
-      </c>
-      <c r="C28" s="38" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="B29" s="37" t="s">
         <v>336</v>
       </c>
-      <c r="B29" s="37" t="s">
+      <c r="C29" s="38" t="s">
         <v>337</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
+        <v>338</v>
+      </c>
+      <c r="B30" s="37" t="s">
         <v>339</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="C30" s="38" t="s">
         <v>340</v>
-      </c>
-      <c r="C30" s="38" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="21" t="s">
+        <v>341</v>
+      </c>
+      <c r="B31" s="37" t="s">
         <v>342</v>
       </c>
-      <c r="B31" s="37" t="s">
+      <c r="C31" s="38" t="s">
         <v>343</v>
-      </c>
-      <c r="C31" s="38" t="s">
-        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -2141,213 +2147,213 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B1" s="6"/>
     </row>
     <row r="3" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="36" t="s">
+        <v>346</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>347</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="30" t="s">
+        <v>348</v>
+      </c>
+      <c r="B6" s="38" t="s">
         <v>349</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
+        <v>350</v>
+      </c>
+      <c r="B7" s="38" t="s">
         <v>351</v>
-      </c>
-      <c r="B7" s="38" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="30" t="s">
+        <v>352</v>
+      </c>
+      <c r="B8" s="38" t="s">
         <v>353</v>
-      </c>
-      <c r="B8" s="38" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="30" t="s">
+        <v>354</v>
+      </c>
+      <c r="B9" s="38" t="s">
         <v>355</v>
-      </c>
-      <c r="B9" s="38" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
+        <v>356</v>
+      </c>
+      <c r="B10" s="38" t="s">
         <v>357</v>
-      </c>
-      <c r="B10" s="38" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="30" t="s">
+        <v>358</v>
+      </c>
+      <c r="B11" s="38" t="s">
         <v>359</v>
-      </c>
-      <c r="B11" s="38" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="30" t="s">
+        <v>360</v>
+      </c>
+      <c r="B12" s="38" t="s">
         <v>361</v>
-      </c>
-      <c r="B12" s="38" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="30" t="s">
+        <v>362</v>
+      </c>
+      <c r="B13" s="38" t="s">
         <v>363</v>
-      </c>
-      <c r="B13" s="38" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="30" t="s">
+        <v>364</v>
+      </c>
+      <c r="B14" s="38" t="s">
         <v>365</v>
-      </c>
-      <c r="B14" s="38" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="30" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="30" t="s">
+        <v>367</v>
+      </c>
+      <c r="B16" s="38" t="s">
         <v>368</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
+        <v>369</v>
+      </c>
+      <c r="B17" s="38" t="s">
         <v>370</v>
-      </c>
-      <c r="B17" s="38" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="30" t="s">
+        <v>371</v>
+      </c>
+      <c r="B18" s="38" t="s">
         <v>372</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="30" t="s">
+        <v>373</v>
+      </c>
+      <c r="B19" s="38" t="s">
         <v>374</v>
-      </c>
-      <c r="B19" s="38" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="30" t="s">
+        <v>375</v>
+      </c>
+      <c r="B20" s="38" t="s">
         <v>376</v>
-      </c>
-      <c r="B20" s="38" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="30" t="s">
+        <v>377</v>
+      </c>
+      <c r="B21" s="38" t="s">
         <v>378</v>
-      </c>
-      <c r="B21" s="38" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="30" t="s">
+        <v>379</v>
+      </c>
+      <c r="B22" s="38" t="s">
         <v>380</v>
-      </c>
-      <c r="B22" s="38" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="30" t="s">
+        <v>381</v>
+      </c>
+      <c r="B23" s="38" t="s">
         <v>382</v>
-      </c>
-      <c r="B23" s="38" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="30" t="s">
+        <v>383</v>
+      </c>
+      <c r="B24" s="38" t="s">
         <v>384</v>
-      </c>
-      <c r="B24" s="38" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="30" t="s">
+        <v>385</v>
+      </c>
+      <c r="B25" s="38" t="s">
         <v>386</v>
-      </c>
-      <c r="B25" s="38" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="30" t="s">
+        <v>387</v>
+      </c>
+      <c r="B26" s="38" t="s">
         <v>388</v>
-      </c>
-      <c r="B26" s="38" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="30" t="s">
+        <v>389</v>
+      </c>
+      <c r="B27" s="38" t="s">
         <v>390</v>
-      </c>
-      <c r="B27" s="38" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="30" t="s">
+        <v>391</v>
+      </c>
+      <c r="B28" s="38" t="s">
         <v>392</v>
-      </c>
-      <c r="B28" s="38" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="30" t="s">
+        <v>393</v>
+      </c>
+      <c r="B29" s="38" t="s">
         <v>394</v>
-      </c>
-      <c r="B29" s="38" t="s">
-        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -7159,7 +7165,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -7219,24 +7225,24 @@
         <v>195</v>
       </c>
       <c r="B7" s="23">
-        <f ca="1">(IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$94,'2015 CARE Projection'!C18:C52,0)),"n/a"))*(1+Inputs!$B$26)^B6+Inputs!$B$43</f>
+        <f ca="1">(IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$94,'2015 CARE Projection'!C18:C52,0)),"n/a"))+Inputs!$B$43</f>
         <v>48708.709380462344</v>
       </c>
       <c r="C7" s="23">
-        <f ca="1">(IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$97,'2015 CARE Projection'!C18:C52,0)),"n/a"))*(1+Inputs!$B$26)^C6+Inputs!$B$43</f>
-        <v>63276.154927676129</v>
+        <f ca="1">(IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$97,'2015 CARE Projection'!C18:C52,0)),"n/a"))+Inputs!$B$43</f>
+        <v>56170.946600652765</v>
       </c>
       <c r="D7" s="23">
-        <f ca="1">(IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$100,'2015 CARE Projection'!C18:C52,0)),"n/a"))*(1+Inputs!$B$26)^D6+Inputs!$B$43</f>
+        <f ca="1">(IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$100,'2015 CARE Projection'!C18:C52,0)),"n/a"))+Inputs!$B$43</f>
         <v>75573.513398167095</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>196</v>
+        <v>397</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B8" s="26">
         <f>MAX(0,1-MAX(0,(Inputs!$B$7-Inputs!$B$95)-Inputs!$B$49)*Inputs!$B$50)</f>
@@ -7251,12 +7257,12 @@
         <v>0.95</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B9" s="23">
         <f ca="1">B7*B8</f>
@@ -7264,7 +7270,7 @@
       </c>
       <c r="C9" s="23">
         <f ca="1">C7*C8</f>
-        <v>63276.154927676129</v>
+        <v>56170.946600652765</v>
       </c>
       <c r="D9" s="23">
         <f ca="1">D7*D8</f>
@@ -7273,7 +7279,7 @@
     </row>
     <row r="10" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B10" s="23">
         <f ca="1">(IF(Inputs!$B$95&gt;=60,'Legacy Scheme'!B6,0)+IF(Inputs!$B$95&gt;=65,'Legacy Scheme'!B10,0))*(IF(Inputs!$B$18="Yes",(1+Inputs!$B$19)^(Inputs!$B$95-Inputs!$B$5),1))</f>
@@ -7288,12 +7294,12 @@
         <v>0</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B11" s="23">
         <f ca="1">(IF(Inputs!$B$95&gt;=60,'Legacy Scheme'!B7,0)+IF(Inputs!$B$95&gt;=65,'Legacy Scheme'!B11,0))*(IF(Inputs!$B$18="Yes",(1+Inputs!$B$19)^(Inputs!$B$95-Inputs!$B$5),1))</f>
@@ -7310,7 +7316,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B12" s="23">
         <f>IF(Inputs!$B$95&gt;=Inputs!$B$7,Inputs!$B$8,0)</f>
@@ -7327,7 +7333,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B13" s="23">
         <f ca="1">IFERROR(INDEX('Private Pensions Projection'!I5:I39,MATCH(Inputs!$B$94,'Private Pensions Projection'!C5:C39,0)),"n/a")</f>
@@ -7344,7 +7350,7 @@
     </row>
     <row r="14" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B14" s="23">
         <f>IF(B6&gt;0,B13/B6,0)</f>
@@ -7359,12 +7365,12 @@
         <v>0</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B15" s="23">
         <f ca="1">IF(B6&gt;0,0,B13)</f>
@@ -7379,12 +7385,12 @@
         <v>887900.41814975906</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B16" s="23">
         <f ca="1">IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",B15*0.04,IF(Inputs!$B$95&gt;=Inputs!$B$7,B15*0.04,B15/MAX(1,Inputs!$B$7-Inputs!$B$95)))</f>
@@ -7399,12 +7405,12 @@
         <v>35516.016725990361</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B17" s="23">
         <f>(IF(Inputs!$B$63="Defined Benefit",IF(Inputs!$B$95&gt;=Inputs!$B$65,Inputs!$B$64,0),0)+IF(Inputs!$B$63="Defined Contribution",IF(Inputs!$B$95&gt;=Inputs!$B$68,(Inputs!$B$66*(1+Inputs!$B$67)^(Inputs!$B$95-Inputs!$B$5))*(IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",0.04,IF(Inputs!$B$95&gt;=Inputs!$B$7,0.04,1/MAX(1,Inputs!$B$7-Inputs!$B$95)))),0),0))+(IF(Inputs!$B$70="Defined Benefit",IF(Inputs!$B$95&gt;=Inputs!$B$72,Inputs!$B$71,0),0)+IF(Inputs!$B$70="Defined Contribution",IF(Inputs!$B$95&gt;=Inputs!$B$75,(Inputs!$B$73*(1+Inputs!$B$74)^(Inputs!$B$95-Inputs!$B$5))*(IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",0.04,IF(Inputs!$B$95&gt;=Inputs!$B$7,0.04,1/MAX(1,Inputs!$B$7-Inputs!$B$95)))),0),0))+(IF(Inputs!$B$77="Defined Benefit",IF(Inputs!$B$95&gt;=Inputs!$B$79,Inputs!$B$78,0),0)+IF(Inputs!$B$77="Defined Contribution",IF(Inputs!$B$95&gt;=Inputs!$B$82,(Inputs!$B$80*(1+Inputs!$B$81)^(Inputs!$B$95-Inputs!$B$5))*(IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",0.04,IF(Inputs!$B$95&gt;=Inputs!$B$7,0.04,1/MAX(1,Inputs!$B$7-Inputs!$B$95)))),0),0))</f>
@@ -7419,7 +7425,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -7430,7 +7436,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="28" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B19" s="29">
         <f ca="1">B9+B10+B12+B16+B17</f>
@@ -7438,7 +7444,7 @@
       </c>
       <c r="C19" s="29">
         <f ca="1">C9+C10+C12+C16+C17</f>
-        <v>75823.754927676127</v>
+        <v>68718.546600652771</v>
       </c>
       <c r="D19" s="29">
         <f ca="1">D9+D10+D12+D16+D17</f>
@@ -7447,7 +7453,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="28" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B20" s="29">
         <f>B14</f>
@@ -7462,12 +7468,12 @@
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="30" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B21" s="31">
         <f ca="1">B11</f>
@@ -7480,6 +7486,26 @@
       <c r="D21" s="31">
         <f ca="1">D11</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="28" t="s">
+        <v>395</v>
+      </c>
+      <c r="B23" s="29">
+        <f ca="1">IF(Inputs!$B$95&gt;=Inputs!$B$7,B19,B19+Inputs!$B$8)</f>
+        <v>52905.143367333563</v>
+      </c>
+      <c r="C23" s="29">
+        <f ca="1">IF(Inputs!$B$98&gt;=Inputs!$B$7,C19,C19+Inputs!$B$8)</f>
+        <v>68718.546600652771</v>
+      </c>
+      <c r="D23" s="29">
+        <f ca="1">IF(Inputs!$B$101&gt;=Inputs!$B$7,D19,D19+Inputs!$B$8)</f>
+        <v>119858.45445424909</v>
+      </c>
+      <c r="E23" t="s">
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -7500,7 +7526,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -7509,7 +7535,7 @@
     </row>
     <row r="3" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="40" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B3" s="40"/>
       <c r="C3" s="40"/>
@@ -7518,7 +7544,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B5" s="22">
         <f>Inputs!$B$105</f>
@@ -7529,7 +7555,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B6" s="23">
         <f>Inputs!$B$104</f>
@@ -7546,7 +7572,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="28" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B8" s="32"/>
       <c r="C8" s="27"/>
@@ -7554,7 +7580,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B9" s="23">
         <f ca="1">(IF(Inputs!$B$105&gt;=60,'Legacy Scheme'!B6,0)+IF(Inputs!$B$105&gt;=65,'Legacy Scheme'!B10,0))*(IF(Inputs!$B$18="Yes",(1+Inputs!$B$19)^(Inputs!$B$105-Inputs!$B$5),1))</f>
@@ -7565,7 +7591,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B10" s="23">
         <f ca="1">IFERROR(INDEX('2015 CARE Projection'!G18:G52,MATCH(Inputs!$B$105,'2015 CARE Projection'!C18:C52,0)),"n/a")+Inputs!$B$43</f>
@@ -7576,7 +7602,7 @@
     </row>
     <row r="11" spans="1:5" ht="36.6" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B11" s="26">
         <f>MAX(0,1-MAX(0,(Inputs!$B$7-Inputs!$B$105)-Inputs!$B$49)*Inputs!$B$50)</f>
@@ -7585,12 +7611,12 @@
       <c r="C11" s="27"/>
       <c r="D11" s="27"/>
       <c r="E11" s="13" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B12" s="23">
         <f ca="1">B10*B11</f>
@@ -7601,7 +7627,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B13" s="23">
         <f>IF(Inputs!$B$105&gt;=Inputs!$B$7,Inputs!$B$8,0)</f>
@@ -7612,7 +7638,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B14" s="23">
         <f>(IF(Inputs!$B$63="Defined Benefit",IF(Inputs!$B$105&gt;=Inputs!$B$65,Inputs!$B$64,0),0)+IF(Inputs!$B$63="Defined Contribution",IF(Inputs!$B$105&gt;=Inputs!$B$68,(Inputs!$B$66*(1+Inputs!$B$67)^(Inputs!$B$105-Inputs!$B$5))*(IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",0.04,IF(Inputs!$B$105&gt;=Inputs!$B$7,0.04,1/MAX(1,Inputs!$B$7-Inputs!$B$105)))),0),0))+(IF(Inputs!$B$70="Defined Benefit",IF(Inputs!$B$105&gt;=Inputs!$B$72,Inputs!$B$71,0),0)+IF(Inputs!$B$70="Defined Contribution",IF(Inputs!$B$105&gt;=Inputs!$B$75,(Inputs!$B$73*(1+Inputs!$B$74)^(Inputs!$B$105-Inputs!$B$5))*(IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",0.04,IF(Inputs!$B$105&gt;=Inputs!$B$7,0.04,1/MAX(1,Inputs!$B$7-Inputs!$B$105)))),0),0))+(IF(Inputs!$B$77="Defined Benefit",IF(Inputs!$B$105&gt;=Inputs!$B$79,Inputs!$B$78,0),0)+IF(Inputs!$B$77="Defined Contribution",IF(Inputs!$B$105&gt;=Inputs!$B$82,(Inputs!$B$80*(1+Inputs!$B$81)^(Inputs!$B$105-Inputs!$B$5))*(IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",0.04,IF(Inputs!$B$105&gt;=Inputs!$B$7,0.04,1/MAX(1,Inputs!$B$7-Inputs!$B$105)))),0),0))</f>
@@ -7623,7 +7649,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="28" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B15" s="29">
         <f ca="1">B9+B12+B13+B14</f>
@@ -7640,7 +7666,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="28" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B17" s="32"/>
       <c r="C17" s="27"/>
@@ -7648,7 +7674,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="21" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B18" s="23">
         <f ca="1">MAX(0,Inputs!$B$104-B15)</f>
@@ -7659,7 +7685,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B19" s="23">
         <f ca="1">IF(Inputs!$B$90="4% Safe Withdrawal (perpetual)",B18/0.04,IF(Inputs!$B$105&gt;=Inputs!$B$7,B18/0.04,B18*MAX(1,Inputs!$B$7-Inputs!$B$105)))</f>
@@ -7668,12 +7694,12 @@
       <c r="C19" s="27"/>
       <c r="D19" s="27"/>
       <c r="E19" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B20" s="23">
         <f ca="1">IFERROR(INDEX('Private Pensions Projection'!I5:I39,MATCH(Inputs!$B$105,'Private Pensions Projection'!C5:C39,0)),"n/a")</f>
@@ -7684,7 +7710,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="28" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B21" s="29">
         <f ca="1">MAX(0,B19-B20)</f>
@@ -7695,7 +7721,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="21" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B22" s="22">
         <f ca="1">MAX(1,Inputs!$B$105-Inputs!$B$5)</f>
@@ -7712,7 +7738,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="28" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="32"/>
@@ -7721,18 +7747,18 @@
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="33"/>
       <c r="B25" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="C25" s="33" t="s">
         <v>238</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="D25" s="33" t="s">
         <v>239</v>
-      </c>
-      <c r="D25" s="33" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B26" s="26">
         <f>MAX(0,Inputs!$B$106-0.015)</f>
@@ -7749,7 +7775,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="30" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B27" s="34">
         <f ca="1">IF(B26=0,B21/B22,B21*B26/((1+B26)^B22-1))</f>
@@ -7766,7 +7792,7 @@
     </row>
     <row r="29" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="39" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39"/>
@@ -7795,7 +7821,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -7804,7 +7830,7 @@
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="41" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
@@ -7813,22 +7839,22 @@
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>246</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="C5" s="20" t="s">
         <v>247</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>248</v>
       </c>
       <c r="D5" s="20"/>
       <c r="E5" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="30" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B6" s="23">
         <v>13900</v>
@@ -7838,12 +7864,12 @@
       </c>
       <c r="D6" s="27"/>
       <c r="E6" s="35" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B7" s="23">
         <v>32700</v>
@@ -7853,12 +7879,12 @@
       </c>
       <c r="D7" s="27"/>
       <c r="E7" s="35" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="30" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B8" s="23">
         <v>45400</v>
@@ -7868,12 +7894,12 @@
       </c>
       <c r="D8" s="27"/>
       <c r="E8" s="35" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="39" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B10" s="39"/>
       <c r="C10" s="39"/>
@@ -7882,7 +7908,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -7891,24 +7917,24 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="33"/>
       <c r="B15" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="33" t="s">
         <v>259</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="D15" s="33" t="s">
         <v>260</v>
-      </c>
-      <c r="D15" s="33" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B16" s="23">
         <f ca="1">'Scenario Summary'!B19</f>
@@ -7916,7 +7942,7 @@
       </c>
       <c r="C16" s="23">
         <f ca="1">'Scenario Summary'!C19</f>
-        <v>75823.754927676127</v>
+        <v>68718.546600652771</v>
       </c>
       <c r="D16" s="23">
         <f ca="1">'Scenario Summary'!D19</f>
@@ -7925,7 +7951,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B17" s="30" t="str">
         <f ca="1">IF(B16&lt;IF(Inputs!$B$109="One-person",B6,C6),"Below Minimum",IF(B16&lt;IF(Inputs!$B$109="One-person",B7,C7),"Minimum",IF(B16&lt;IF(Inputs!$B$109="One-person",B8,C8),"Moderate","Comfortable")))</f>

</xml_diff>